<commit_message>
feat: Robot de revisión automática de campañas y reportes administrativos
Reescribe descargar_campanas.js: navega directo a Reportes Promotor, cubre las campañas y reportes actuales (incluyendo Educar es Creer, Poder de Elegirte, Convenciones Promotores, Pagado/Pendiente), compara fecha de corte contra lo ya desplegado antes de tocar nada, y solo procesa/despliega/notifica lo que realmente cambió. Lo que no cambió se descarta.

Agrega deploy_datos.sh (deploy de solo datos a N carpetas, reutilizable). Renombra EDUCAR ES CREER -> educar_es_creer para evitar el bug de rsync viejo de macOS con espacios en rutas remotas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/administrador/pagado_emitidido/pagado_emitido_reclutas.xlsx
+++ b/administrador/pagado_emitidido/pagado_emitido_reclutas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>7 de agosto de 2026</t>
+          <t>15 de septiembre de 2026</t>
         </is>
       </c>
       <c r="B1" t="inlineStr"/>
@@ -487,13 +487,13 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>2396.76</v>
+        <v>16207.97</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2396.76</v>
+        <v>16207.97</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -502,16 +502,16 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>26364.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>118915</t>
+          <t>120051</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -521,7 +521,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>HUMBERTO EMMANUEL SANDOVAL MOLINS</t>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -539,16 +539,188 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>2623.27</v>
       </c>
       <c r="L5" t="n">
-        <v>49020.81</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>49020.81</v>
+        <v>2623.27</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>119223</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OSCAR RAMIREZ RUIZ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>12054.68</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>12054.68</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>38468.95</v>
+      </c>
+      <c r="M6" t="n">
+        <v>38468.95</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>120051</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GUILLERMO JOSE RAMIREZ RAMIREZ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2488.17</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2488.17</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>27369.85</v>
+      </c>
+      <c r="M7" t="n">
+        <v>27369.85</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>119447</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1742.89</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1742.89</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>71981.92</v>
+      </c>
+      <c r="M8" t="n">
+        <v>71981.92</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>116795</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2043</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GERARDO DANIEL BARAJAS TORRES</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4796.14</v>
+      </c>
+      <c r="M9" t="n">
+        <v>4796.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>